<commit_message>
data: publish heavy LinkTask link-prediction report (GCN)
Regenerate results/link-prediction-gcn/ from the heavy AMLT rerun
(epochs=50, task_num=3 folds, All-in-one caps 128/1/24), replacing the
earlier under-fit fast report.

Improvements vs fast run:
- Degenerate AUROC=0.5 cells: 43 -> 13 (epochs 10->50 fixed under-fitting;
  remaining 13 are genuine constant-predictor cases on PROTEINS/MUTAG).
- Cells with real std: 0 -> 2901 / 2912 (task_num 1->3 yields mean+/-std).
- AUROC median 0.6482 -> 0.6719, max 0.9507; full coverage (2912 combos).

Also prune empty Graph/Node/Link placeholder matrices that were never
populated by the link-only sweep, and add a Run configuration note to the
report README.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/results/link-prediction-gcn/Link/0shot/CiteSeer/GCN_total_results.xlsx
+++ b/results/link-prediction-gcn/Link/0shot/CiteSeer/GCN_total_results.xlsx
@@ -893,457 +893,457 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>0.5451±0.0584</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0.4780±0.0141</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0.4692±0.0009</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0.4429±0.0000</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>0.4692±0.0000</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.6766±0.0064</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>0.7026±0.0041</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>0.7026±0.0041</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>0.7026±0.0041</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0.6810±0.0180</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>0.6908±0.0149</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.7059±0.0091</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>0.6659±0.0000</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>0.6659±0.0000</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>0.6659±0.0000</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>0.4923±0.0153</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>0.4952±0.0136</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>0.5835±0.0000</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0.6747±0.0000</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>0.7117±0.0049</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>0.4703±0.0000</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>0.4890±0.0000</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>0.6385±0.0000</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>0.7238±0.0160</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>0.7000±0.0080</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
+        <is>
+          <t>0.5590±0.0432</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>0.4872±0.0159</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>0.5128±0.0132</t>
+        </is>
+      </c>
+      <c r="AF2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>0.6659±0.0000</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>0.6879±0.0000</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>0.6212±0.0873</t>
+        </is>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>0.7432±0.0075</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
+          <t>0.7432±0.0075</t>
+        </is>
+      </c>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>0.7432±0.0075</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>0.6227±0.0877</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>0.7150±0.0063</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>0.7392±0.0166</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AP2" t="inlineStr">
+        <is>
+          <t>0.6432±0.0858</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>0.4897±0.0427</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>0.5000±0.0326</t>
+        </is>
+      </c>
+      <c r="AS2" t="inlineStr">
+        <is>
+          <t>0.4993±0.0010</t>
+        </is>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>0.4985±0.0021</t>
+        </is>
+      </c>
+      <c r="AU2" t="inlineStr">
+        <is>
+          <t>0.7205±0.0143</t>
+        </is>
+      </c>
+      <c r="AV2" t="inlineStr">
+        <is>
+          <t>0.6139±0.0338</t>
+        </is>
+      </c>
+      <c r="AW2" t="inlineStr">
+        <is>
+          <t>0.6139±0.0338</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>0.6139±0.0338</t>
+        </is>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>0.7172±0.0143</t>
+        </is>
+      </c>
+      <c r="AZ2" t="inlineStr">
+        <is>
+          <t>0.6916±0.0215</t>
+        </is>
+      </c>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>0.6227±0.0021</t>
+        </is>
+      </c>
+      <c r="BB2" t="inlineStr">
+        <is>
+          <t>0.5062±0.0060</t>
+        </is>
+      </c>
+      <c r="BC2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>0.4407±0.0000</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>0.4462±0.0000</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
+      <c r="BD2" t="inlineStr">
+        <is>
+          <t>0.5341±0.0115</t>
+        </is>
+      </c>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>0.5311±0.0029</t>
+        </is>
+      </c>
+      <c r="BF2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="BG2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>0.6132±0.0823</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>0.6872±0.0275</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>0.6872±0.0275</t>
+        </is>
+      </c>
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>0.6872±0.0275</t>
+        </is>
+      </c>
+      <c r="BL2" t="inlineStr">
+        <is>
+          <t>0.6114±0.0796</t>
+        </is>
+      </c>
+      <c r="BM2" t="inlineStr">
+        <is>
+          <t>0.6260±0.0381</t>
+        </is>
+      </c>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>0.6853±0.0104</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>0.5297±0.0000</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>0.5297±0.0000</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>0.5297±0.0000</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
+      <c r="BP2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>0.6033±0.0000</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>0.5484±0.0000</t>
-        </is>
-      </c>
-      <c r="AO2" t="inlineStr">
+      <c r="BQ2" t="inlineStr">
+        <is>
+          <t>0.4626±0.0018</t>
+        </is>
+      </c>
+      <c r="BR2" t="inlineStr">
+        <is>
+          <t>0.5527±0.0102</t>
+        </is>
+      </c>
+      <c r="BS2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AP2" t="inlineStr">
-        <is>
-          <t>0.5824±0.0000</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr">
-        <is>
-          <t>0.4615±0.0000</t>
-        </is>
-      </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>0.4846±0.0000</t>
-        </is>
-      </c>
-      <c r="AS2" t="inlineStr">
+      <c r="BT2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AT2" t="inlineStr">
+      <c r="BU2" t="inlineStr">
+        <is>
+          <t>0.5480±0.0679</t>
+        </is>
+      </c>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>0.7110±0.0142</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>0.7165±0.0179</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr">
+        <is>
+          <t>0.7007±0.0181</t>
+        </is>
+      </c>
+      <c r="BY2" t="inlineStr">
+        <is>
+          <t>0.5491±0.0694</t>
+        </is>
+      </c>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>0.6890±0.0139</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>0.7293±0.0066</t>
+        </is>
+      </c>
+      <c r="CB2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="AU2" t="inlineStr">
-        <is>
-          <t>0.6055±0.0000</t>
-        </is>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t>0.6802±0.0000</t>
-        </is>
-      </c>
-      <c r="AW2" t="inlineStr">
-        <is>
-          <t>0.6802±0.0000</t>
-        </is>
-      </c>
-      <c r="AX2" t="inlineStr">
-        <is>
-          <t>0.6802±0.0000</t>
-        </is>
-      </c>
-      <c r="AY2" t="inlineStr">
-        <is>
-          <t>0.6560±0.0000</t>
-        </is>
-      </c>
-      <c r="AZ2" t="inlineStr">
-        <is>
-          <t>0.6473±0.0000</t>
-        </is>
-      </c>
-      <c r="BA2" t="inlineStr">
-        <is>
-          <t>0.6769±0.0000</t>
-        </is>
-      </c>
-      <c r="BB2" t="inlineStr">
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>0.7216±0.0060</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>0.5037±0.0108</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr">
+        <is>
+          <t>0.5059±0.0076</t>
+        </is>
+      </c>
+      <c r="CF2" t="inlineStr">
         <is>
           <t>0.5000±0.0000</t>
         </is>
       </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BD2" t="inlineStr">
-        <is>
-          <t>0.4945±0.0000</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
-        <is>
-          <t>0.4648±0.0000</t>
-        </is>
-      </c>
-      <c r="BF2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>0.5484±0.0000</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr">
-        <is>
-          <t>0.5484±0.0000</t>
-        </is>
-      </c>
-      <c r="BK2" t="inlineStr">
-        <is>
-          <t>0.5484±0.0000</t>
-        </is>
-      </c>
-      <c r="BL2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BM2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>0.6637±0.0000</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BP2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BQ2" t="inlineStr">
-        <is>
-          <t>0.4989±0.0000</t>
-        </is>
-      </c>
-      <c r="BR2" t="inlineStr">
-        <is>
-          <t>0.4604±0.0000</t>
-        </is>
-      </c>
-      <c r="BS2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BT2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BU2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>0.6154±0.0000</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>0.6154±0.0000</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr">
-        <is>
-          <t>0.6154±0.0000</t>
-        </is>
-      </c>
-      <c r="BY2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr">
-        <is>
-          <t>0.6692±0.0000</t>
-        </is>
-      </c>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr">
-        <is>
-          <t>0.4626±0.0000</t>
-        </is>
-      </c>
-      <c r="CE2" t="inlineStr">
-        <is>
-          <t>0.4462±0.0000</t>
-        </is>
-      </c>
-      <c r="CF2" t="inlineStr">
-        <is>
-          <t>0.5000±0.0000</t>
-        </is>
-      </c>
       <c r="CG2" t="inlineStr">
         <is>
-          <t>0.5000±0.0000</t>
+          <t>0.4993±0.0010</t>
         </is>
       </c>
       <c r="CH2" t="inlineStr">
         <is>
-          <t>0.5198±0.0000</t>
+          <t>0.7179±0.0101</t>
         </is>
       </c>
       <c r="CI2" t="inlineStr">
         <is>
-          <t>0.5242±0.0000</t>
+          <t>0.5187±0.0041</t>
         </is>
       </c>
       <c r="CJ2" t="inlineStr">
         <is>
-          <t>0.5242±0.0000</t>
+          <t>0.5187±0.0041</t>
         </is>
       </c>
       <c r="CK2" t="inlineStr">
         <is>
-          <t>0.5242±0.0000</t>
+          <t>0.5187±0.0041</t>
         </is>
       </c>
       <c r="CL2" t="inlineStr">
         <is>
-          <t>0.5099±0.0000</t>
+          <t>0.5813±0.1049</t>
         </is>
       </c>
       <c r="CM2" t="inlineStr">
         <is>
-          <t>0.6615±0.0000</t>
+          <t>0.6564±0.0165</t>
         </is>
       </c>
       <c r="CN2" t="inlineStr">
         <is>
-          <t>0.5253±0.0000</t>
+          <t>0.5158±0.0054</t>
         </is>
       </c>
     </row>
@@ -1355,457 +1355,457 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>0.4301±0.2761</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0.6355±0.0231</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.6032±0.0064</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0.5967±0.0000</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0.6305±0.0000</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.7284±0.0060</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0.7534±0.0060</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0.7534±0.0060</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0.7534±0.0060</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0.7311±0.0172</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0.7389±0.0114</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0.7557±0.0078</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0.7305±0.0000</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0.7305±0.0000</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0.7305±0.0000</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>0.6302±0.0156</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0.6480±0.0118</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0.6408±0.0000</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0.7381±0.0000</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>0.7660±0.0032</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>0.6269±0.0000</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>0.6420±0.0000</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>0.7270±0.0000</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>0.7713±0.0117</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>0.7513±0.0066</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>0.6774±0.0076</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>0.6252±0.0266</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0.6303±0.0074</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>0.7384±0.0000</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>0.7418±0.0000</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>0.0000±0.0000</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AH3" t="inlineStr">
+        <is>
+          <t>0.7092±0.0340</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>0.7906±0.0054</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>0.7906±0.0054</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>0.7906±0.0054</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>0.7108±0.0334</t>
+        </is>
+      </c>
+      <c r="AM3" t="inlineStr">
+        <is>
+          <t>0.7673±0.0072</t>
+        </is>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>0.7870±0.0112</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
+        <is>
+          <t>0.4444±0.3143</t>
+        </is>
+      </c>
+      <c r="AP3" t="inlineStr">
+        <is>
+          <t>0.7288±0.0369</t>
+        </is>
+      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>0.6322±0.0339</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr">
+        <is>
+          <t>0.6351±0.0198</t>
+        </is>
+      </c>
+      <c r="AS3" t="inlineStr">
+        <is>
+          <t>0.6657±0.0014</t>
+        </is>
+      </c>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>0.6654±0.0018</t>
+        </is>
+      </c>
+      <c r="AU3" t="inlineStr">
+        <is>
+          <t>0.7692±0.0099</t>
+        </is>
+      </c>
+      <c r="AV3" t="inlineStr">
+        <is>
+          <t>0.7191±0.0165</t>
+        </is>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>0.7191±0.0165</t>
+        </is>
+      </c>
+      <c r="AX3" t="inlineStr">
+        <is>
+          <t>0.7191±0.0165</t>
+        </is>
+      </c>
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>0.7663±0.0101</t>
+        </is>
+      </c>
+      <c r="AZ3" t="inlineStr">
+        <is>
+          <t>0.7479±0.0084</t>
+        </is>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>0.7224±0.0013</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>0.2466±0.2975</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>0.5925±0.0000</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>0.5902±0.0000</t>
-        </is>
-      </c>
-      <c r="AF3" t="inlineStr">
+      <c r="BD3" t="inlineStr">
+        <is>
+          <t>0.6279±0.0083</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>0.6268±0.0027</t>
+        </is>
+      </c>
+      <c r="BF3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="BG3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>0.7037±0.0307</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>0.7374±0.0234</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>0.7374±0.0234</t>
+        </is>
+      </c>
+      <c r="BK3" t="inlineStr">
+        <is>
+          <t>0.7374±0.0234</t>
+        </is>
+      </c>
+      <c r="BL3" t="inlineStr">
+        <is>
+          <t>0.7032±0.0282</t>
+        </is>
+      </c>
+      <c r="BM3" t="inlineStr">
+        <is>
+          <t>0.7196±0.0184</t>
+        </is>
+      </c>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>0.7374±0.0072</t>
+        </is>
+      </c>
+      <c r="BO3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>0.6787±0.0000</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
-        <is>
-          <t>0.6787±0.0000</t>
-        </is>
-      </c>
-      <c r="AK3" t="inlineStr">
-        <is>
-          <t>0.6787±0.0000</t>
-        </is>
-      </c>
-      <c r="AL3" t="inlineStr">
+      <c r="BP3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>0.7110±0.0000</t>
-        </is>
-      </c>
-      <c r="AN3" t="inlineStr">
-        <is>
-          <t>0.6826±0.0000</t>
-        </is>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>0.0000±0.0000</t>
-        </is>
-      </c>
-      <c r="AP3" t="inlineStr">
-        <is>
-          <t>0.6998±0.0000</t>
-        </is>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>0.6184±0.0000</t>
-        </is>
-      </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>0.6455±0.0000</t>
-        </is>
-      </c>
-      <c r="AS3" t="inlineStr">
+      <c r="BQ3" t="inlineStr">
+        <is>
+          <t>0.6053±0.0098</t>
+        </is>
+      </c>
+      <c r="BR3" t="inlineStr">
+        <is>
+          <t>0.6380±0.0044</t>
+        </is>
+      </c>
+      <c r="BS3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AT3" t="inlineStr">
+      <c r="BT3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="AU3" t="inlineStr">
-        <is>
-          <t>0.7103±0.0000</t>
-        </is>
-      </c>
-      <c r="AV3" t="inlineStr">
-        <is>
-          <t>0.7436±0.0000</t>
-        </is>
-      </c>
-      <c r="AW3" t="inlineStr">
-        <is>
-          <t>0.7436±0.0000</t>
-        </is>
-      </c>
-      <c r="AX3" t="inlineStr">
-        <is>
-          <t>0.7436±0.0000</t>
-        </is>
-      </c>
-      <c r="AY3" t="inlineStr">
-        <is>
-          <t>0.7304±0.0000</t>
-        </is>
-      </c>
-      <c r="AZ3" t="inlineStr">
-        <is>
-          <t>0.7230±0.0000</t>
-        </is>
-      </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>0.7421±0.0000</t>
-        </is>
-      </c>
-      <c r="BB3" t="inlineStr">
-        <is>
-          <t>0.0000±0.0000</t>
-        </is>
-      </c>
-      <c r="BC3" t="inlineStr">
+      <c r="BU3" t="inlineStr">
+        <is>
+          <t>0.6780±0.0160</t>
+        </is>
+      </c>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>0.7624±0.0120</t>
+        </is>
+      </c>
+      <c r="BW3" t="inlineStr">
+        <is>
+          <t>0.7674±0.0163</t>
+        </is>
+      </c>
+      <c r="BX3" t="inlineStr">
+        <is>
+          <t>0.7549±0.0153</t>
+        </is>
+      </c>
+      <c r="BY3" t="inlineStr">
+        <is>
+          <t>0.6790±0.0174</t>
+        </is>
+      </c>
+      <c r="BZ3" t="inlineStr">
+        <is>
+          <t>0.7425±0.0068</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr">
+        <is>
+          <t>0.7792±0.0059</t>
+        </is>
+      </c>
+      <c r="CB3" t="inlineStr">
+        <is>
+          <t>0.4444±0.3143</t>
+        </is>
+      </c>
+      <c r="CC3" t="inlineStr">
+        <is>
+          <t>0.7741±0.0051</t>
+        </is>
+      </c>
+      <c r="CD3" t="inlineStr">
+        <is>
+          <t>0.6485±0.0069</t>
+        </is>
+      </c>
+      <c r="CE3" t="inlineStr">
+        <is>
+          <t>0.6593±0.0076</t>
+        </is>
+      </c>
+      <c r="CF3" t="inlineStr">
         <is>
           <t>0.6667±0.0000</t>
         </is>
       </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>0.6618±0.0000</t>
-        </is>
-      </c>
-      <c r="BE3" t="inlineStr">
-        <is>
-          <t>0.6268±0.0000</t>
-        </is>
-      </c>
-      <c r="BF3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BH3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BI3" t="inlineStr">
-        <is>
-          <t>0.6746±0.0000</t>
-        </is>
-      </c>
-      <c r="BJ3" t="inlineStr">
-        <is>
-          <t>0.6746±0.0000</t>
-        </is>
-      </c>
-      <c r="BK3" t="inlineStr">
-        <is>
-          <t>0.6746±0.0000</t>
-        </is>
-      </c>
-      <c r="BL3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BM3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BN3" t="inlineStr">
-        <is>
-          <t>0.7177±0.0000</t>
-        </is>
-      </c>
-      <c r="BO3" t="inlineStr">
-        <is>
-          <t>0.0000±0.0000</t>
-        </is>
-      </c>
-      <c r="BP3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BQ3" t="inlineStr">
-        <is>
-          <t>0.6657±0.0000</t>
-        </is>
-      </c>
-      <c r="BR3" t="inlineStr">
-        <is>
-          <t>0.6185±0.0000</t>
-        </is>
-      </c>
-      <c r="BS3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BT3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BU3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BV3" t="inlineStr">
-        <is>
-          <t>0.7059±0.0000</t>
-        </is>
-      </c>
-      <c r="BW3" t="inlineStr">
-        <is>
-          <t>0.7059±0.0000</t>
-        </is>
-      </c>
-      <c r="BX3" t="inlineStr">
-        <is>
-          <t>0.7059±0.0000</t>
-        </is>
-      </c>
-      <c r="BY3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="BZ3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="CA3" t="inlineStr">
-        <is>
-          <t>0.7300±0.0000</t>
-        </is>
-      </c>
-      <c r="CB3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="CC3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
-      <c r="CD3" t="inlineStr">
-        <is>
-          <t>0.6134±0.0000</t>
-        </is>
-      </c>
-      <c r="CE3" t="inlineStr">
-        <is>
-          <t>0.5902±0.0000</t>
-        </is>
-      </c>
-      <c r="CF3" t="inlineStr">
-        <is>
-          <t>0.6667±0.0000</t>
-        </is>
-      </c>
       <c r="CG3" t="inlineStr">
         <is>
-          <t>0.6667±0.0000</t>
+          <t>0.6660±0.0009</t>
         </is>
       </c>
       <c r="CH3" t="inlineStr">
         <is>
-          <t>0.6756±0.0000</t>
+          <t>0.7694±0.0073</t>
         </is>
       </c>
       <c r="CI3" t="inlineStr">
         <is>
-          <t>0.6776±0.0000</t>
+          <t>0.6749±0.0017</t>
         </is>
       </c>
       <c r="CJ3" t="inlineStr">
         <is>
-          <t>0.6776±0.0000</t>
+          <t>0.6749±0.0017</t>
         </is>
       </c>
       <c r="CK3" t="inlineStr">
         <is>
-          <t>0.6776±0.0000</t>
+          <t>0.6749±0.0017</t>
         </is>
       </c>
       <c r="CL3" t="inlineStr">
         <is>
-          <t>0.6711±0.0000</t>
+          <t>0.7067±0.0521</t>
         </is>
       </c>
       <c r="CM3" t="inlineStr">
         <is>
-          <t>0.7381±0.0000</t>
+          <t>0.7396±0.0057</t>
         </is>
       </c>
       <c r="CN3" t="inlineStr">
         <is>
-          <t>0.6776±0.0000</t>
+          <t>0.6736±0.0023</t>
         </is>
       </c>
     </row>
@@ -1817,457 +1817,457 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.5785±0.0000</t>
+          <t>0.5973±0.0110</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.6831±0.0000</t>
+          <t>0.6836±0.0179</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.5797±0.0000</t>
+          <t>0.6132±0.0104</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.5982±0.0000</t>
+          <t>0.6478±0.0069</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.6666±0.0000</t>
+          <t>0.6754±0.0095</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.7015±0.0000</t>
+          <t>0.7271±0.0199</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.6820±0.0000</t>
+          <t>0.7899±0.0070</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.8074±0.0000</t>
+          <t>0.8132±0.0167</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>0.8074±0.0000</t>
+          <t>0.8132±0.0167</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>0.8074±0.0000</t>
+          <t>0.8132±0.0167</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0.6884±0.0000</t>
+          <t>0.7884±0.0127</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.6510±0.0000</t>
+          <t>0.8126±0.0091</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.8098±0.0000</t>
+          <t>0.8117±0.0158</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.5090±0.0000</t>
+          <t>0.6008±0.0722</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0.7303±0.0000</t>
+          <t>0.7408±0.0141</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0.6452±0.0000</t>
+          <t>0.6709±0.0245</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>0.6774±0.0000</t>
+          <t>0.7153±0.0307</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>0.6415±0.0000</t>
+          <t>0.6480±0.0190</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>0.6277±0.0000</t>
+          <t>0.6424±0.0186</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>0.8389±0.0000</t>
+          <t>0.8559±0.0095</t>
         </is>
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>0.7240±0.0000</t>
+          <t>0.7383±0.0158</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>0.7240±0.0000</t>
+          <t>0.7383±0.0158</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>0.7240±0.0000</t>
+          <t>0.7383±0.0158</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>0.8433±0.0000</t>
+          <t>0.8632±0.0109</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>0.7824±0.0000</t>
+          <t>0.7960±0.0105</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>0.7492±0.0000</t>
+          <t>0.7610±0.0100</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
         <is>
-          <t>0.4625±0.0000</t>
+          <t>0.5560±0.0400</t>
         </is>
       </c>
       <c r="AC4" t="inlineStr">
         <is>
-          <t>0.6407±0.0000</t>
+          <t>0.6874±0.0223</t>
         </is>
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>0.5989±0.0000</t>
+          <t>0.6265±0.0175</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>0.6019±0.0000</t>
+          <t>0.6810±0.0244</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
         <is>
-          <t>0.6453±0.0000</t>
+          <t>0.6450±0.0192</t>
         </is>
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>0.6441±0.0000</t>
+          <t>0.6584±0.0135</t>
         </is>
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>0.6679±0.0000</t>
+          <t>0.7438±0.0639</t>
         </is>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>0.7055±0.0000</t>
+          <t>0.8922±0.0160</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>0.7055±0.0000</t>
+          <t>0.8922±0.0160</t>
         </is>
       </c>
       <c r="AK4" t="inlineStr">
         <is>
-          <t>0.7055±0.0000</t>
+          <t>0.8922±0.0160</t>
         </is>
       </c>
       <c r="AL4" t="inlineStr">
         <is>
-          <t>0.6649±0.0000</t>
+          <t>0.7466±0.0628</t>
         </is>
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>0.8416±0.0000</t>
+          <t>0.8672±0.0111</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>0.7033±0.0000</t>
+          <t>0.8844±0.0025</t>
         </is>
       </c>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>0.5752±0.0000</t>
+          <t>0.6132±0.0223</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr">
         <is>
-          <t>0.7237±0.0000</t>
+          <t>0.8153±0.0186</t>
         </is>
       </c>
       <c r="AQ4" t="inlineStr">
         <is>
-          <t>0.5682±0.0000</t>
+          <t>0.6962±0.0413</t>
         </is>
       </c>
       <c r="AR4" t="inlineStr">
         <is>
-          <t>0.6591±0.0000</t>
+          <t>0.6789±0.0203</t>
         </is>
       </c>
       <c r="AS4" t="inlineStr">
         <is>
-          <t>0.6730±0.0000</t>
+          <t>0.6646±0.0166</t>
         </is>
       </c>
       <c r="AT4" t="inlineStr">
         <is>
-          <t>0.6333±0.0000</t>
+          <t>0.6505±0.0225</t>
         </is>
       </c>
       <c r="AU4" t="inlineStr">
         <is>
-          <t>0.7439±0.0000</t>
+          <t>0.8500±0.0074</t>
         </is>
       </c>
       <c r="AV4" t="inlineStr">
         <is>
-          <t>0.7918±0.0000</t>
+          <t>0.7933±0.0163</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>0.7918±0.0000</t>
+          <t>0.7933±0.0163</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>0.7918±0.0000</t>
+          <t>0.7933±0.0163</t>
         </is>
       </c>
       <c r="AY4" t="inlineStr">
         <is>
-          <t>0.7587±0.0000</t>
+          <t>0.8481±0.0076</t>
         </is>
       </c>
       <c r="AZ4" t="inlineStr">
         <is>
-          <t>0.7751±0.0000</t>
+          <t>0.8120±0.0052</t>
         </is>
       </c>
       <c r="BA4" t="inlineStr">
         <is>
-          <t>0.7875±0.0000</t>
+          <t>0.7881±0.0139</t>
         </is>
       </c>
       <c r="BB4" t="inlineStr">
         <is>
-          <t>0.6276±0.0000</t>
+          <t>0.6282±0.0076</t>
         </is>
       </c>
       <c r="BC4" t="inlineStr">
         <is>
-          <t>0.6393±0.0000</t>
+          <t>0.6723±0.0108</t>
         </is>
       </c>
       <c r="BD4" t="inlineStr">
         <is>
-          <t>0.5951±0.0000</t>
+          <t>0.6490±0.0117</t>
         </is>
       </c>
       <c r="BE4" t="inlineStr">
         <is>
-          <t>0.5982±0.0000</t>
+          <t>0.6919±0.0117</t>
         </is>
       </c>
       <c r="BF4" t="inlineStr">
         <is>
-          <t>0.6442±0.0000</t>
+          <t>0.6462±0.0068</t>
         </is>
       </c>
       <c r="BG4" t="inlineStr">
         <is>
-          <t>0.6447±0.0000</t>
+          <t>0.6441±0.0165</t>
         </is>
       </c>
       <c r="BH4" t="inlineStr">
         <is>
-          <t>0.6608±0.0000</t>
+          <t>0.7440±0.0577</t>
         </is>
       </c>
       <c r="BI4" t="inlineStr">
         <is>
-          <t>0.6944±0.0000</t>
+          <t>0.7862±0.0309</t>
         </is>
       </c>
       <c r="BJ4" t="inlineStr">
         <is>
-          <t>0.6944±0.0000</t>
+          <t>0.7862±0.0309</t>
         </is>
       </c>
       <c r="BK4" t="inlineStr">
         <is>
-          <t>0.6944±0.0000</t>
+          <t>0.7862±0.0309</t>
         </is>
       </c>
       <c r="BL4" t="inlineStr">
         <is>
-          <t>0.6657±0.0000</t>
+          <t>0.7432±0.0535</t>
         </is>
       </c>
       <c r="BM4" t="inlineStr">
         <is>
-          <t>0.7022±0.0000</t>
+          <t>0.8537±0.0054</t>
         </is>
       </c>
       <c r="BN4" t="inlineStr">
         <is>
-          <t>0.7540±0.0000</t>
+          <t>0.7890±0.0115</t>
         </is>
       </c>
       <c r="BO4" t="inlineStr">
         <is>
-          <t>0.5794±0.0000</t>
+          <t>0.5876±0.0304</t>
         </is>
       </c>
       <c r="BP4" t="inlineStr">
         <is>
-          <t>0.6482±0.0000</t>
+          <t>0.6730±0.0197</t>
         </is>
       </c>
       <c r="BQ4" t="inlineStr">
         <is>
-          <t>0.5959±0.0000</t>
+          <t>0.6163±0.0134</t>
         </is>
       </c>
       <c r="BR4" t="inlineStr">
         <is>
-          <t>0.5990±0.0000</t>
+          <t>0.6840±0.0089</t>
         </is>
       </c>
       <c r="BS4" t="inlineStr">
         <is>
-          <t>0.6411±0.0000</t>
+          <t>0.6662±0.0175</t>
         </is>
       </c>
       <c r="BT4" t="inlineStr">
         <is>
-          <t>0.6461±0.0000</t>
+          <t>0.6417±0.0072</t>
         </is>
       </c>
       <c r="BU4" t="inlineStr">
         <is>
-          <t>0.6525±0.0000</t>
+          <t>0.7098±0.0266</t>
         </is>
       </c>
       <c r="BV4" t="inlineStr">
         <is>
-          <t>0.7369±0.0000</t>
+          <t>0.8253±0.0155</t>
         </is>
       </c>
       <c r="BW4" t="inlineStr">
         <is>
-          <t>0.7369±0.0000</t>
+          <t>0.8296±0.0208</t>
         </is>
       </c>
       <c r="BX4" t="inlineStr">
         <is>
-          <t>0.7369±0.0000</t>
+          <t>0.8186±0.0298</t>
         </is>
       </c>
       <c r="BY4" t="inlineStr">
         <is>
-          <t>0.6593±0.0000</t>
+          <t>0.7137±0.0395</t>
         </is>
       </c>
       <c r="BZ4" t="inlineStr">
         <is>
-          <t>0.6634±0.0000</t>
+          <t>0.8390±0.0054</t>
         </is>
       </c>
       <c r="CA4" t="inlineStr">
         <is>
-          <t>0.7554±0.0000</t>
+          <t>0.8626±0.0038</t>
         </is>
       </c>
       <c r="CB4" t="inlineStr">
         <is>
-          <t>0.5236±0.0000</t>
+          <t>0.5591±0.0395</t>
         </is>
       </c>
       <c r="CC4" t="inlineStr">
         <is>
-          <t>0.7419±0.0000</t>
+          <t>0.8523±0.0149</t>
         </is>
       </c>
       <c r="CD4" t="inlineStr">
         <is>
-          <t>0.4656±0.0000</t>
+          <t>0.7072±0.0054</t>
         </is>
       </c>
       <c r="CE4" t="inlineStr">
         <is>
-          <t>0.4870±0.0000</t>
+          <t>0.7440±0.0202</t>
         </is>
       </c>
       <c r="CF4" t="inlineStr">
         <is>
-          <t>0.6398±0.0000</t>
+          <t>0.6382±0.0227</t>
         </is>
       </c>
       <c r="CG4" t="inlineStr">
         <is>
-          <t>0.5554±0.0000</t>
+          <t>0.6362±0.0268</t>
         </is>
       </c>
       <c r="CH4" t="inlineStr">
         <is>
-          <t>0.7632±0.0000</t>
+          <t>0.8539±0.0076</t>
         </is>
       </c>
       <c r="CI4" t="inlineStr">
         <is>
-          <t>0.7058±0.0000</t>
+          <t>0.7669±0.0099</t>
         </is>
       </c>
       <c r="CJ4" t="inlineStr">
         <is>
-          <t>0.7058±0.0000</t>
+          <t>0.7669±0.0099</t>
         </is>
       </c>
       <c r="CK4" t="inlineStr">
         <is>
-          <t>0.7058±0.0000</t>
+          <t>0.7669±0.0099</t>
         </is>
       </c>
       <c r="CL4" t="inlineStr">
         <is>
-          <t>0.7423±0.0000</t>
+          <t>0.7989±0.0498</t>
         </is>
       </c>
       <c r="CM4" t="inlineStr">
         <is>
-          <t>0.7968±0.0000</t>
+          <t>0.8289±0.0126</t>
         </is>
       </c>
       <c r="CN4" t="inlineStr">
         <is>
-          <t>0.6962±0.0000</t>
+          <t>0.7550±0.0093</t>
         </is>
       </c>
     </row>
@@ -2279,457 +2279,457 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.6179±0.0000</t>
+          <t>0.6536±0.0211</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.7158±0.0000</t>
+          <t>0.7213±0.0174</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.6179±0.0000</t>
+          <t>0.6961±0.0082</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.6857±0.0000</t>
+          <t>0.7157±0.0055</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.6916±0.0000</t>
+          <t>0.6938±0.0014</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.7296±0.0000</t>
+          <t>0.7483±0.0153</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.7178±0.0000</t>
+          <t>0.7996±0.0098</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.8114±0.0000</t>
+          <t>0.8153±0.0170</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0.8114±0.0000</t>
+          <t>0.8153±0.0170</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>0.8114±0.0000</t>
+          <t>0.8153±0.0170</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0.7215±0.0000</t>
+          <t>0.7986±0.0122</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.6980±0.0000</t>
+          <t>0.8281±0.0088</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.8121±0.0000</t>
+          <t>0.8125±0.0158</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.5545±0.0000</t>
+          <t>0.6554±0.0754</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0.7446±0.0000</t>
+          <t>0.7519±0.0081</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>0.6811±0.0000</t>
+          <t>0.7089±0.0370</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>0.7197±0.0000</t>
+          <t>0.7472±0.0244</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>0.6517±0.0000</t>
+          <t>0.6686±0.0174</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>0.6676±0.0000</t>
+          <t>0.6730±0.0077</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>0.8443±0.0000</t>
+          <t>0.8550±0.0106</t>
         </is>
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>0.7193±0.0000</t>
+          <t>0.7321±0.0096</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>0.7193±0.0000</t>
+          <t>0.7321±0.0096</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>0.7193±0.0000</t>
+          <t>0.7321±0.0096</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>0.8468±0.0000</t>
+          <t>0.8634±0.0115</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>0.7577±0.0000</t>
+          <t>0.7704±0.0107</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>0.7496±0.0000</t>
+          <t>0.7540±0.0035</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>0.5408±0.0000</t>
+          <t>0.6261±0.0378</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>0.6627±0.0000</t>
+          <t>0.7258±0.0265</t>
         </is>
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>0.6875±0.0000</t>
+          <t>0.7026±0.0092</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>0.6868±0.0000</t>
+          <t>0.7399±0.0197</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
         <is>
-          <t>0.6623±0.0000</t>
+          <t>0.6641±0.0147</t>
         </is>
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>0.6652±0.0000</t>
+          <t>0.6747±0.0106</t>
         </is>
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>0.6956±0.0000</t>
+          <t>0.7619±0.0432</t>
         </is>
       </c>
       <c r="AI5" t="inlineStr">
         <is>
-          <t>0.7393±0.0000</t>
+          <t>0.8896±0.0142</t>
         </is>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>0.7393±0.0000</t>
+          <t>0.8896±0.0142</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr">
         <is>
-          <t>0.7393±0.0000</t>
+          <t>0.8896±0.0142</t>
         </is>
       </c>
       <c r="AL5" t="inlineStr">
         <is>
-          <t>0.6952±0.0000</t>
+          <t>0.7652±0.0403</t>
         </is>
       </c>
       <c r="AM5" t="inlineStr">
         <is>
-          <t>0.8488±0.0000</t>
+          <t>0.8670±0.0080</t>
         </is>
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>0.7349±0.0000</t>
+          <t>0.8805±0.0037</t>
         </is>
       </c>
       <c r="AO5" t="inlineStr">
         <is>
-          <t>0.6470±0.0000</t>
+          <t>0.6738±0.0324</t>
         </is>
       </c>
       <c r="AP5" t="inlineStr">
         <is>
-          <t>0.7143±0.0000</t>
+          <t>0.8168±0.0212</t>
         </is>
       </c>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>0.5751±0.0000</t>
+          <t>0.7436±0.0267</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
         <is>
-          <t>0.7101±0.0000</t>
+          <t>0.6938±0.0174</t>
         </is>
       </c>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>0.6851±0.0000</t>
+          <t>0.6881±0.0189</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
         <is>
-          <t>0.6540±0.0000</t>
+          <t>0.6718±0.0190</t>
         </is>
       </c>
       <c r="AU5" t="inlineStr">
         <is>
-          <t>0.7358±0.0000</t>
+          <t>0.8520±0.0032</t>
         </is>
       </c>
       <c r="AV5" t="inlineStr">
         <is>
-          <t>0.7919±0.0000</t>
+          <t>0.7494±0.0276</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>0.7919±0.0000</t>
+          <t>0.7494±0.0276</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>0.7919±0.0000</t>
+          <t>0.7494±0.0276</t>
         </is>
       </c>
       <c r="AY5" t="inlineStr">
         <is>
-          <t>0.7568±0.0000</t>
+          <t>0.8520±0.0037</t>
         </is>
       </c>
       <c r="AZ5" t="inlineStr">
         <is>
-          <t>0.7455±0.0000</t>
+          <t>0.7846±0.0103</t>
         </is>
       </c>
       <c r="BA5" t="inlineStr">
         <is>
-          <t>0.7817±0.0000</t>
+          <t>0.7430±0.0174</t>
         </is>
       </c>
       <c r="BB5" t="inlineStr">
         <is>
-          <t>0.6728±0.0000</t>
+          <t>0.6878±0.0119</t>
         </is>
       </c>
       <c r="BC5" t="inlineStr">
         <is>
-          <t>0.6605±0.0000</t>
+          <t>0.7041±0.0111</t>
         </is>
       </c>
       <c r="BD5" t="inlineStr">
         <is>
-          <t>0.6827±0.0000</t>
+          <t>0.7114±0.0074</t>
         </is>
       </c>
       <c r="BE5" t="inlineStr">
         <is>
-          <t>0.6884±0.0000</t>
+          <t>0.7550±0.0080</t>
         </is>
       </c>
       <c r="BF5" t="inlineStr">
         <is>
-          <t>0.6627±0.0000</t>
+          <t>0.6709±0.0059</t>
         </is>
       </c>
       <c r="BG5" t="inlineStr">
         <is>
-          <t>0.6633±0.0000</t>
+          <t>0.6665±0.0079</t>
         </is>
       </c>
       <c r="BH5" t="inlineStr">
         <is>
-          <t>0.6884±0.0000</t>
+          <t>0.7617±0.0444</t>
         </is>
       </c>
       <c r="BI5" t="inlineStr">
         <is>
-          <t>0.7341±0.0000</t>
+          <t>0.7916±0.0259</t>
         </is>
       </c>
       <c r="BJ5" t="inlineStr">
         <is>
-          <t>0.7341±0.0000</t>
+          <t>0.7916±0.0259</t>
         </is>
       </c>
       <c r="BK5" t="inlineStr">
         <is>
-          <t>0.7341±0.0000</t>
+          <t>0.7916±0.0259</t>
         </is>
       </c>
       <c r="BL5" t="inlineStr">
         <is>
-          <t>0.6964±0.0000</t>
+          <t>0.7558±0.0381</t>
         </is>
       </c>
       <c r="BM5" t="inlineStr">
         <is>
-          <t>0.7578±0.0000</t>
+          <t>0.8685±0.0071</t>
         </is>
       </c>
       <c r="BN5" t="inlineStr">
         <is>
-          <t>0.7602±0.0000</t>
+          <t>0.7930±0.0151</t>
         </is>
       </c>
       <c r="BO5" t="inlineStr">
         <is>
-          <t>0.6226±0.0000</t>
+          <t>0.6365±0.0365</t>
         </is>
       </c>
       <c r="BP5" t="inlineStr">
         <is>
-          <t>0.6390±0.0000</t>
+          <t>0.6540±0.0137</t>
         </is>
       </c>
       <c r="BQ5" t="inlineStr">
         <is>
-          <t>0.6848±0.0000</t>
+          <t>0.6975±0.0074</t>
         </is>
       </c>
       <c r="BR5" t="inlineStr">
         <is>
-          <t>0.6862±0.0000</t>
+          <t>0.7439±0.0082</t>
         </is>
       </c>
       <c r="BS5" t="inlineStr">
         <is>
-          <t>0.6597±0.0000</t>
+          <t>0.6866±0.0196</t>
         </is>
       </c>
       <c r="BT5" t="inlineStr">
         <is>
-          <t>0.6633±0.0000</t>
+          <t>0.6621±0.0010</t>
         </is>
       </c>
       <c r="BU5" t="inlineStr">
         <is>
-          <t>0.6764±0.0000</t>
+          <t>0.7294±0.0260</t>
         </is>
       </c>
       <c r="BV5" t="inlineStr">
         <is>
-          <t>0.7527±0.0000</t>
+          <t>0.8287±0.0129</t>
         </is>
       </c>
       <c r="BW5" t="inlineStr">
         <is>
-          <t>0.7527±0.0000</t>
+          <t>0.8313±0.0160</t>
         </is>
       </c>
       <c r="BX5" t="inlineStr">
         <is>
-          <t>0.7527±0.0000</t>
+          <t>0.8221±0.0296</t>
         </is>
       </c>
       <c r="BY5" t="inlineStr">
         <is>
-          <t>0.6814±0.0000</t>
+          <t>0.7354±0.0314</t>
         </is>
       </c>
       <c r="BZ5" t="inlineStr">
         <is>
-          <t>0.7401±0.0000</t>
+          <t>0.8626±0.0020</t>
         </is>
       </c>
       <c r="CA5" t="inlineStr">
         <is>
-          <t>0.7606±0.0000</t>
+          <t>0.8597±0.0081</t>
         </is>
       </c>
       <c r="CB5" t="inlineStr">
         <is>
-          <t>0.5713±0.0000</t>
+          <t>0.6251±0.0428</t>
         </is>
       </c>
       <c r="CC5" t="inlineStr">
         <is>
-          <t>0.7370±0.0000</t>
+          <t>0.8491±0.0148</t>
         </is>
       </c>
       <c r="CD5" t="inlineStr">
         <is>
-          <t>0.4829±0.0000</t>
+          <t>0.7457±0.0036</t>
         </is>
       </c>
       <c r="CE5" t="inlineStr">
         <is>
-          <t>0.4971±0.0000</t>
+          <t>0.7547±0.0160</t>
         </is>
       </c>
       <c r="CF5" t="inlineStr">
         <is>
-          <t>0.6599±0.0000</t>
+          <t>0.6551±0.0144</t>
         </is>
       </c>
       <c r="CG5" t="inlineStr">
         <is>
-          <t>0.5885±0.0000</t>
+          <t>0.6566±0.0263</t>
         </is>
       </c>
       <c r="CH5" t="inlineStr">
         <is>
-          <t>0.7471±0.0000</t>
+          <t>0.8535±0.0058</t>
         </is>
       </c>
       <c r="CI5" t="inlineStr">
         <is>
-          <t>0.6586±0.0000</t>
+          <t>0.7178±0.0141</t>
         </is>
       </c>
       <c r="CJ5" t="inlineStr">
         <is>
-          <t>0.6586±0.0000</t>
+          <t>0.7178±0.0141</t>
         </is>
       </c>
       <c r="CK5" t="inlineStr">
         <is>
-          <t>0.6586±0.0000</t>
+          <t>0.7178±0.0141</t>
         </is>
       </c>
       <c r="CL5" t="inlineStr">
         <is>
-          <t>0.7288±0.0000</t>
+          <t>0.7877±0.0554</t>
         </is>
       </c>
       <c r="CM5" t="inlineStr">
         <is>
-          <t>0.7662±0.0000</t>
+          <t>0.8101±0.0166</t>
         </is>
       </c>
       <c r="CN5" t="inlineStr">
         <is>
-          <t>0.6379±0.0000</t>
+          <t>0.7028±0.0131</t>
         </is>
       </c>
     </row>

</xml_diff>